<commit_message>
Update error processing and Excel reports
Changed the 'ORIGEM DO ERRO' field for missing segment status errors in processamento_erros.py to 'Atualização de Trechos'. Updated several Excel report files to reflect recent data or structural changes.
</commit_message>
<xml_diff>
--- a/Integration Quality/EMPRESAS/Relatorio - KONTRIP VIAGENS.xlsx
+++ b/Integration Quality/EMPRESAS/Relatorio - KONTRIP VIAGENS.xlsx
@@ -18,7 +18,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +41,9 @@
     <font>
       <b val="1"/>
       <color rgb="00591F6A"/>
+    </font>
+    <font>
+      <color rgb="00FF0000"/>
     </font>
   </fonts>
   <fills count="4">
@@ -90,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -106,6 +109,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -711,14 +717,14 @@
       <c r="E2" s="6" t="n">
         <v>45842.79048611111</v>
       </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>24 a 31 dias</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>24 a 31 dias</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
@@ -902,14 +908,14 @@
       <c r="E3" s="6" t="n">
         <v>45842.63230324074</v>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>24 a 31 dias</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>24 a 31 dias</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">

</xml_diff>